<commit_message>
RSP json type data extracted mapped in fron end. BSP in progress
</commit_message>
<xml_diff>
--- a/Report_format/Monthly/technopara may-2026.xlsx
+++ b/Report_format/Monthly/technopara may-2026.xlsx
@@ -1,11 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9302"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFA88403-CB0F-4B52-828E-27C07902FE96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12036" yWindow="2136" windowWidth="10800" windowHeight="9924" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7920" yWindow="660" windowWidth="14910" windowHeight="10590"/>
   </bookViews>
   <sheets>
     <sheet name="PAGE-1-8" sheetId="1" r:id="rId1"/>
@@ -19,7 +18,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="0">'PAGE-1-8'!$A$1:$AM$348</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'page-9'!$A$1:$R$45</definedName>
   </definedNames>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="144525"/>
 </workbook>
 </file>
 
@@ -1487,7 +1486,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.00_)"/>
@@ -2036,8 +2035,8 @@
   <cellStyles count="5">
     <cellStyle name="Good" xfId="3" builtinId="26"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
-    <cellStyle name="Normal 5" xfId="4" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
+    <cellStyle name="Normal 2" xfId="1"/>
+    <cellStyle name="Normal 5" xfId="4"/>
     <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -2054,9 +2053,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2094,7 +2093,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -2166,7 +2165,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2339,28 +2338,28 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A2:EU364"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="18" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="48.88671875" style="97" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.6640625" style="68" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="48.85546875" style="97" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.7109375" style="68" bestFit="1" customWidth="1"/>
     <col min="3" max="17" width="0" style="68" hidden="1" customWidth="1"/>
-    <col min="18" max="18" width="12.44140625" style="68" customWidth="1"/>
+    <col min="18" max="18" width="12.42578125" style="68" hidden="1" customWidth="1"/>
     <col min="19" max="19" width="13" style="68" customWidth="1"/>
     <col min="20" max="20" width="18" style="68" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="13.6640625" style="68" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="11.6640625" style="68" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="16.33203125" style="100" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="16.33203125" style="68" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="13.7109375" style="68" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="11.7109375" style="68" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="16.28515625" style="100" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="16.28515625" style="68" bestFit="1" customWidth="1"/>
     <col min="25" max="38" width="0" style="68" hidden="1" customWidth="1"/>
-    <col min="39" max="39" width="13.6640625" style="68" bestFit="1" customWidth="1"/>
-    <col min="40" max="52" width="9.109375" style="66"/>
-    <col min="53" max="61" width="9.109375" style="60"/>
-    <col min="62" max="16384" width="9.109375" style="66"/>
+    <col min="39" max="39" width="13.7109375" style="68" bestFit="1" customWidth="1"/>
+    <col min="40" max="52" width="9.140625" style="66"/>
+    <col min="53" max="61" width="9.140625" style="60"/>
+    <col min="62" max="16384" width="9.140625" style="66"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:61" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -2418,7 +2417,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="3" spans="1:61" s="68" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:61" s="68" customFormat="1" ht="18" x14ac:dyDescent="0.35">
       <c r="A3" s="67" t="s">
         <v>142</v>
       </c>
@@ -2564,7 +2563,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="4" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A4" s="69" t="s">
         <v>178</v>
       </c>
@@ -2643,7 +2642,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="5" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A5" s="62" t="s">
         <v>180</v>
       </c>
@@ -2762,7 +2761,7 @@
         <v>75.999861959088122</v>
       </c>
     </row>
-    <row r="6" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A6" s="62" t="s">
         <v>182</v>
       </c>
@@ -2881,7 +2880,7 @@
         <v>11.025131368517249</v>
       </c>
     </row>
-    <row r="7" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A7" s="62" t="s">
         <v>182</v>
       </c>
@@ -3000,7 +2999,7 @@
         <v>69.390002962127909</v>
       </c>
     </row>
-    <row r="8" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A8" s="62" t="s">
         <v>185</v>
       </c>
@@ -3119,7 +3118,7 @@
         <v>10.787571395933288</v>
       </c>
     </row>
-    <row r="9" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A9" s="62" t="s">
         <v>185</v>
       </c>
@@ -3238,7 +3237,7 @@
         <v>67.894847335379026</v>
       </c>
     </row>
-    <row r="10" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A10" s="62" t="s">
         <v>186</v>
       </c>
@@ -3357,7 +3356,7 @@
         <v>320.03693252679295</v>
       </c>
     </row>
-    <row r="11" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A11" s="62" t="s">
         <v>188</v>
       </c>
@@ -3476,7 +3475,7 @@
         <v>15.888645190769934</v>
       </c>
     </row>
-    <row r="12" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A12" s="62" t="s">
         <v>189</v>
       </c>
@@ -3595,7 +3594,7 @@
         <v>86.209952713826596</v>
       </c>
     </row>
-    <row r="13" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A13" s="62" t="s">
         <v>190</v>
       </c>
@@ -3712,7 +3711,7 @@
         <v>7.0750000000000002</v>
       </c>
     </row>
-    <row r="14" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A14" s="62" t="s">
         <v>191</v>
       </c>
@@ -3831,7 +3830,7 @@
         <v>4248.4139161462981</v>
       </c>
     </row>
-    <row r="15" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A15" s="62" t="s">
         <v>193</v>
       </c>
@@ -3950,7 +3949,7 @@
         <v>5.25</v>
       </c>
     </row>
-    <row r="16" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A16" s="69" t="s">
         <v>194</v>
       </c>
@@ -3993,7 +3992,7 @@
       <c r="AL16" s="6"/>
       <c r="AM16" s="6"/>
     </row>
-    <row r="17" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A17" s="62" t="s">
         <v>188</v>
       </c>
@@ -4100,7 +4099,7 @@
         <v>30.32407577708295</v>
       </c>
     </row>
-    <row r="18" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A18" s="62" t="s">
         <v>180</v>
       </c>
@@ -4207,7 +4206,7 @@
         <v>76.000169828715613</v>
       </c>
     </row>
-    <row r="19" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A19" s="62" t="s">
         <v>180</v>
       </c>
@@ -4314,7 +4313,7 @@
         <v>23.046349089571454</v>
       </c>
     </row>
-    <row r="20" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A20" s="62" t="s">
         <v>195</v>
       </c>
@@ -4421,7 +4420,7 @@
         <v>20.103733676659921</v>
       </c>
     </row>
-    <row r="21" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A21" s="62" t="s">
         <v>185</v>
       </c>
@@ -4528,7 +4527,7 @@
         <v>66.296278325003641</v>
       </c>
     </row>
-    <row r="22" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A22" s="62" t="s">
         <v>196</v>
       </c>
@@ -4635,7 +4634,7 @@
         <v>2.9426154129115321</v>
       </c>
     </row>
-    <row r="23" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A23" s="62" t="s">
         <v>196</v>
       </c>
@@ -4742,7 +4741,7 @@
         <v>9.7038915037119704</v>
       </c>
     </row>
-    <row r="24" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A24" s="62" t="s">
         <v>189</v>
       </c>
@@ -4849,7 +4848,7 @@
         <v>87.994536156319242</v>
       </c>
     </row>
-    <row r="25" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A25" s="62" t="s">
         <v>190</v>
       </c>
@@ -4952,7 +4951,7 @@
         <v>5.7050000000000001</v>
       </c>
     </row>
-    <row r="26" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A26" s="71" t="s">
         <v>197</v>
       </c>
@@ -4995,7 +4994,7 @@
       <c r="AL26" s="5"/>
       <c r="AM26" s="5"/>
     </row>
-    <row r="27" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A27" s="62" t="s">
         <v>198</v>
       </c>
@@ -5112,7 +5111,7 @@
         <v>3.1957003092109755</v>
       </c>
     </row>
-    <row r="28" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A28" s="62" t="s">
         <v>199</v>
       </c>
@@ -5229,7 +5228,7 @@
         <v>0.25653781250304819</v>
       </c>
     </row>
-    <row r="29" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A29" s="62" t="s">
         <v>200</v>
       </c>
@@ -5346,7 +5345,7 @@
         <v>367.08860759493672</v>
       </c>
     </row>
-    <row r="30" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A30" s="62" t="s">
         <v>203</v>
       </c>
@@ -5463,7 +5462,7 @@
         <v>1857.0342205323193</v>
       </c>
     </row>
-    <row r="31" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A31" s="62" t="s">
         <v>204</v>
       </c>
@@ -5550,7 +5549,7 @@
         <v>14.27</v>
       </c>
     </row>
-    <row r="32" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A32" s="62"/>
       <c r="B32" s="5"/>
       <c r="C32" s="5"/>
@@ -5593,7 +5592,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="33" spans="1:61" s="68" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:61" s="68" customFormat="1" ht="18" x14ac:dyDescent="0.35">
       <c r="A33" s="71" t="s">
         <v>206</v>
       </c>
@@ -5721,7 +5720,7 @@
       <c r="BH33" s="60"/>
       <c r="BI33" s="60"/>
     </row>
-    <row r="34" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A34" s="62" t="s">
         <v>208</v>
       </c>
@@ -5838,7 +5837,7 @@
         <v>10.135</v>
       </c>
     </row>
-    <row r="35" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A35" s="62" t="s">
         <v>209</v>
       </c>
@@ -5955,7 +5954,7 @@
         <v>53.28</v>
       </c>
     </row>
-    <row r="36" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A36" s="62" t="s">
         <v>210</v>
       </c>
@@ -6072,7 +6071,7 @@
         <v>10.989999999999998</v>
       </c>
     </row>
-    <row r="37" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A37" s="62" t="s">
         <v>211</v>
       </c>
@@ -6187,7 +6186,7 @@
         <v>1.5750000000000002</v>
       </c>
     </row>
-    <row r="38" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A38" s="62" t="s">
         <v>212</v>
       </c>
@@ -6306,7 +6305,7 @@
         <v>0.73372713031230685</v>
       </c>
     </row>
-    <row r="39" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A39" s="62" t="s">
         <v>214</v>
       </c>
@@ -6425,7 +6424,7 @@
         <v>857.3611219932618</v>
       </c>
     </row>
-    <row r="40" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A40" s="62" t="s">
         <v>216</v>
       </c>
@@ -6544,7 +6543,7 @@
         <v>137.85943743633942</v>
       </c>
     </row>
-    <row r="41" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A41" s="62" t="s">
         <v>217</v>
       </c>
@@ -6663,7 +6662,7 @@
         <v>107.54524798244927</v>
       </c>
     </row>
-    <row r="42" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A42" s="62" t="s">
         <v>218</v>
       </c>
@@ -6782,7 +6781,7 @@
         <v>1.8765180600172373</v>
       </c>
     </row>
-    <row r="43" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A43" s="62" t="s">
         <v>219</v>
       </c>
@@ -6901,7 +6900,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A44" s="62" t="s">
         <v>220</v>
       </c>
@@ -7020,7 +7019,7 @@
         <v>103.41220716132571</v>
       </c>
     </row>
-    <row r="45" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A45" s="62" t="s">
         <v>221</v>
       </c>
@@ -7139,7 +7138,7 @@
         <v>64.032750920629951</v>
       </c>
     </row>
-    <row r="46" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A46" s="62"/>
       <c r="B46" s="5"/>
       <c r="C46" s="7"/>
@@ -7180,7 +7179,7 @@
       <c r="AL46" s="7"/>
       <c r="AM46" s="7"/>
     </row>
-    <row r="47" spans="1:61" s="74" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:61" s="74" customFormat="1" ht="18" x14ac:dyDescent="0.35">
       <c r="A47" s="73" t="s">
         <v>222</v>
       </c>
@@ -7272,7 +7271,7 @@
       <c r="BH47" s="60"/>
       <c r="BI47" s="60"/>
     </row>
-    <row r="48" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A48" s="62" t="s">
         <v>223</v>
       </c>
@@ -7389,7 +7388,7 @@
         <v>96.872955099199444</v>
       </c>
     </row>
-    <row r="49" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A49" s="62" t="s">
         <v>225</v>
       </c>
@@ -7506,7 +7505,7 @@
         <v>87.835000000000008</v>
       </c>
     </row>
-    <row r="50" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A50" s="62" t="s">
         <v>227</v>
       </c>
@@ -7623,7 +7622,7 @@
         <v>82.36</v>
       </c>
     </row>
-    <row r="51" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A51" s="62" t="s">
         <v>228</v>
       </c>
@@ -7740,7 +7739,7 @@
         <v>72.33</v>
       </c>
     </row>
-    <row r="52" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A52" s="62" t="s">
         <v>229</v>
       </c>
@@ -7857,7 +7856,7 @@
         <v>18.577624068128298</v>
       </c>
     </row>
-    <row r="53" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A53" s="71" t="s">
         <v>230</v>
       </c>
@@ -7900,7 +7899,7 @@
       <c r="AL53" s="5"/>
       <c r="AM53" s="5"/>
     </row>
-    <row r="54" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A54" s="62" t="s">
         <v>208</v>
       </c>
@@ -8017,7 +8016,7 @@
         <v>9.92</v>
       </c>
     </row>
-    <row r="55" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A55" s="62" t="s">
         <v>209</v>
       </c>
@@ -8134,7 +8133,7 @@
         <v>53.655000000000001</v>
       </c>
     </row>
-    <row r="56" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A56" s="62" t="s">
         <v>210</v>
       </c>
@@ -8251,7 +8250,7 @@
         <v>10.559999999999999</v>
       </c>
     </row>
-    <row r="57" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A57" s="62" t="s">
         <v>211</v>
       </c>
@@ -8368,7 +8367,7 @@
         <v>1.59</v>
       </c>
     </row>
-    <row r="58" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A58" s="62" t="s">
         <v>212</v>
       </c>
@@ -8487,7 +8486,7 @@
         <v>1.3041048132321993</v>
       </c>
     </row>
-    <row r="59" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A59" s="62" t="s">
         <v>214</v>
       </c>
@@ -8606,7 +8605,7 @@
         <v>765.11559242965541</v>
       </c>
     </row>
-    <row r="60" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A60" s="75" t="s">
         <v>231</v>
       </c>
@@ -8695,7 +8694,7 @@
         <v>88.172074758628824</v>
       </c>
     </row>
-    <row r="61" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A61" s="75" t="s">
         <v>232</v>
       </c>
@@ -8814,7 +8813,7 @@
         <v>95.243437952109602</v>
       </c>
     </row>
-    <row r="62" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A62" s="62" t="s">
         <v>220</v>
       </c>
@@ -8933,7 +8932,7 @@
         <v>262.12760931825562</v>
       </c>
     </row>
-    <row r="63" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A63" s="62" t="s">
         <v>221</v>
       </c>
@@ -9052,7 +9051,7 @@
         <v>63.214148631491923</v>
       </c>
     </row>
-    <row r="64" spans="1:61" s="74" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:61" s="74" customFormat="1" ht="18" x14ac:dyDescent="0.35">
       <c r="A64" s="73" t="s">
         <v>222</v>
       </c>
@@ -9144,7 +9143,7 @@
       <c r="BH64" s="60"/>
       <c r="BI64" s="60"/>
     </row>
-    <row r="65" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A65" s="62" t="s">
         <v>233</v>
       </c>
@@ -9263,7 +9262,7 @@
         <v>13.121143228320882</v>
       </c>
     </row>
-    <row r="66" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A66" s="62" t="s">
         <v>218</v>
       </c>
@@ -9382,7 +9381,7 @@
         <v>2.1819362839174468</v>
       </c>
     </row>
-    <row r="67" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A67" s="62" t="s">
         <v>219</v>
       </c>
@@ -9501,7 +9500,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A68" s="62" t="s">
         <v>234</v>
       </c>
@@ -9618,7 +9617,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A69" s="62" t="s">
         <v>223</v>
       </c>
@@ -9735,7 +9734,7 @@
         <v>95.140495867768607</v>
       </c>
     </row>
-    <row r="70" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A70" s="62" t="s">
         <v>235</v>
       </c>
@@ -9852,7 +9851,7 @@
         <v>85.705000000000013</v>
       </c>
     </row>
-    <row r="71" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A71" s="62" t="s">
         <v>236</v>
       </c>
@@ -9969,7 +9968,7 @@
         <v>75.239999999999995</v>
       </c>
     </row>
-    <row r="72" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A72" s="62" t="s">
         <v>228</v>
       </c>
@@ -10086,7 +10085,7 @@
         <v>74.33</v>
       </c>
     </row>
-    <row r="73" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A73" s="62" t="s">
         <v>229</v>
       </c>
@@ -10203,7 +10202,7 @@
         <v>9.6971685382129724</v>
       </c>
     </row>
-    <row r="74" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A74" s="62"/>
       <c r="B74" s="5"/>
       <c r="C74" s="5"/>
@@ -10246,7 +10245,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="75" spans="1:61" s="68" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:61" s="68" customFormat="1" ht="18" x14ac:dyDescent="0.35">
       <c r="A75" s="62"/>
       <c r="B75" s="5" t="s">
         <v>143</v>
@@ -10372,7 +10371,7 @@
       <c r="BH75" s="60"/>
       <c r="BI75" s="60"/>
     </row>
-    <row r="76" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A76" s="76" t="s">
         <v>238</v>
       </c>
@@ -10415,7 +10414,7 @@
       <c r="AL76" s="5"/>
       <c r="AM76" s="5"/>
     </row>
-    <row r="77" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A77" s="62" t="s">
         <v>208</v>
       </c>
@@ -10518,7 +10517,7 @@
         <v>9.9750000000000014</v>
       </c>
     </row>
-    <row r="78" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A78" s="62" t="s">
         <v>209</v>
       </c>
@@ -10621,7 +10620,7 @@
         <v>53.7</v>
       </c>
     </row>
-    <row r="79" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A79" s="62" t="s">
         <v>210</v>
       </c>
@@ -10724,7 +10723,7 @@
         <v>10.545</v>
       </c>
     </row>
-    <row r="80" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A80" s="62" t="s">
         <v>211</v>
       </c>
@@ -10827,7 +10826,7 @@
         <v>1.59</v>
       </c>
     </row>
-    <row r="81" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A81" s="62" t="s">
         <v>212</v>
       </c>
@@ -10932,7 +10931,7 @@
         <v>1.2809830216288813</v>
       </c>
     </row>
-    <row r="82" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A82" s="62" t="s">
         <v>214</v>
       </c>
@@ -11037,7 +11036,7 @@
         <v>756.7381901715687</v>
       </c>
     </row>
-    <row r="83" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A83" s="62" t="s">
         <v>216</v>
       </c>
@@ -11142,7 +11141,7 @@
         <v>81.213500165872773</v>
       </c>
     </row>
-    <row r="84" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A84" s="62" t="s">
         <v>217</v>
       </c>
@@ -11247,7 +11246,7 @@
         <v>81.474828024361386</v>
       </c>
     </row>
-    <row r="85" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A85" s="62" t="s">
         <v>220</v>
       </c>
@@ -11352,7 +11351,7 @@
         <v>252.29248690231032</v>
       </c>
     </row>
-    <row r="86" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A86" s="62" t="s">
         <v>221</v>
       </c>
@@ -11457,7 +11456,7 @@
         <v>59.222689517466719</v>
       </c>
     </row>
-    <row r="87" spans="1:61" s="74" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:61" s="74" customFormat="1" ht="18" x14ac:dyDescent="0.35">
       <c r="A87" s="73" t="s">
         <v>222</v>
       </c>
@@ -11549,7 +11548,7 @@
       <c r="BH87" s="60"/>
       <c r="BI87" s="60"/>
     </row>
-    <row r="88" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A88" s="62" t="s">
         <v>233</v>
       </c>
@@ -11654,7 +11653,7 @@
         <v>23.203410093827653</v>
       </c>
     </row>
-    <row r="89" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A89" s="62" t="s">
         <v>218</v>
       </c>
@@ -11729,7 +11728,7 @@
         <v>2.1313086422844125</v>
       </c>
     </row>
-    <row r="90" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A90" s="62" t="s">
         <v>219</v>
       </c>
@@ -11832,7 +11831,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A91" s="62" t="s">
         <v>223</v>
       </c>
@@ -11935,7 +11934,7 @@
         <v>97.725669957686875</v>
       </c>
     </row>
-    <row r="92" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A92" s="62" t="s">
         <v>228</v>
       </c>
@@ -12038,7 +12037,7 @@
         <v>74.61</v>
       </c>
     </row>
-    <row r="93" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A93" s="62" t="s">
         <v>229</v>
       </c>
@@ -12141,7 +12140,7 @@
         <v>14.596216593745556</v>
       </c>
     </row>
-    <row r="94" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A94" s="62"/>
       <c r="B94" s="5"/>
       <c r="C94" s="15"/>
@@ -12182,7 +12181,7 @@
       <c r="AL94" s="15"/>
       <c r="AM94" s="15"/>
     </row>
-    <row r="95" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A95" s="62"/>
       <c r="B95" s="5"/>
       <c r="C95" s="15"/>
@@ -12223,7 +12222,7 @@
       <c r="AL95" s="15"/>
       <c r="AM95" s="15"/>
     </row>
-    <row r="96" spans="1:61" s="68" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:61" s="68" customFormat="1" ht="18" x14ac:dyDescent="0.35">
       <c r="A96" s="71" t="s">
         <v>239</v>
       </c>
@@ -12351,7 +12350,7 @@
       <c r="BH96" s="60"/>
       <c r="BI96" s="60"/>
     </row>
-    <row r="97" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A97" s="62" t="s">
         <v>241</v>
       </c>
@@ -12452,7 +12451,7 @@
         <v>1.9043688530630918</v>
       </c>
     </row>
-    <row r="98" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A98" s="62" t="s">
         <v>243</v>
       </c>
@@ -12535,7 +12534,7 @@
       <c r="AL98" s="72"/>
       <c r="AM98" s="72"/>
     </row>
-    <row r="99" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A99" s="62" t="s">
         <v>244</v>
       </c>
@@ -12642,7 +12641,7 @@
         <v>2.6830476341183593</v>
       </c>
     </row>
-    <row r="100" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A100" s="62" t="s">
         <v>245</v>
       </c>
@@ -12757,7 +12756,7 @@
         <v>2.4459834967682723</v>
       </c>
     </row>
-    <row r="101" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A101" s="62" t="s">
         <v>246</v>
       </c>
@@ -12852,7 +12851,7 @@
         <v>449.20060983801909</v>
       </c>
     </row>
-    <row r="102" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A102" s="62" t="s">
         <v>248</v>
       </c>
@@ -12911,7 +12910,7 @@
       <c r="AL102" s="7"/>
       <c r="AM102" s="7"/>
     </row>
-    <row r="103" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A103" s="62" t="s">
         <v>249</v>
       </c>
@@ -13006,7 +13005,7 @@
         <v>377.00845301481183</v>
       </c>
     </row>
-    <row r="104" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A104" s="62" t="s">
         <v>250</v>
       </c>
@@ -13125,7 +13124,7 @@
         <v>394.1188443160782</v>
       </c>
     </row>
-    <row r="105" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A105" s="62" t="s">
         <v>251</v>
       </c>
@@ -13222,7 +13221,7 @@
         <v>111.96135356001706</v>
       </c>
     </row>
-    <row r="106" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A106" s="62" t="s">
         <v>252</v>
       </c>
@@ -13327,7 +13326,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="107" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A107" s="62" t="s">
         <v>254</v>
       </c>
@@ -13432,7 +13431,7 @@
         <v>156.2573723427808</v>
       </c>
     </row>
-    <row r="108" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A108" s="62" t="s">
         <v>255</v>
       </c>
@@ -13535,7 +13534,7 @@
         <v>145.7578447023769</v>
       </c>
     </row>
-    <row r="109" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A109" s="62" t="s">
         <v>256</v>
       </c>
@@ -13606,7 +13605,7 @@
       <c r="AL109" s="80"/>
       <c r="AM109" s="80"/>
     </row>
-    <row r="110" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A110" s="62" t="s">
         <v>257</v>
       </c>
@@ -13677,7 +13676,7 @@
       <c r="AL110" s="80"/>
       <c r="AM110" s="80"/>
     </row>
-    <row r="111" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A111" s="62" t="s">
         <v>258</v>
       </c>
@@ -13774,7 +13773,7 @@
         <v>21.246865053008278</v>
       </c>
     </row>
-    <row r="112" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A112" s="62" t="s">
         <v>259</v>
       </c>
@@ -13893,7 +13892,7 @@
         <v>16.210700336038347</v>
       </c>
     </row>
-    <row r="113" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A113" s="62" t="s">
         <v>260</v>
       </c>
@@ -14012,7 +14011,7 @@
         <v>0.90500000000000003</v>
       </c>
     </row>
-    <row r="114" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A114" s="62" t="s">
         <v>261</v>
       </c>
@@ -14131,7 +14130,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="115" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A115" s="62" t="s">
         <v>262</v>
       </c>
@@ -14250,7 +14249,7 @@
         <v>1286.684878551283</v>
       </c>
     </row>
-    <row r="116" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A116" s="62" t="s">
         <v>263</v>
       </c>
@@ -14369,7 +14368,7 @@
         <v>198.51461912192502</v>
       </c>
     </row>
-    <row r="117" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A117" s="62" t="s">
         <v>264</v>
       </c>
@@ -14468,7 +14467,7 @@
         <v>1331.3819940490612</v>
       </c>
     </row>
-    <row r="118" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A118" s="62" t="s">
         <v>265</v>
       </c>
@@ -14569,7 +14568,7 @@
         <v>1730.2693429737249</v>
       </c>
     </row>
-    <row r="119" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A119" s="62" t="s">
         <v>266</v>
       </c>
@@ -14658,7 +14657,7 @@
         <v>1714.1029493007161</v>
       </c>
     </row>
-    <row r="120" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A120" s="75" t="s">
         <v>267</v>
       </c>
@@ -14763,7 +14762,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A121" s="75" t="s">
         <v>268</v>
       </c>
@@ -14868,7 +14867,7 @@
         <v>245.06984530051687</v>
       </c>
     </row>
-    <row r="122" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A122" s="62" t="s">
         <v>269</v>
       </c>
@@ -14987,7 +14986,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A123" s="62" t="s">
         <v>270</v>
       </c>
@@ -15106,7 +15105,7 @@
         <v>4.8405029360087175</v>
       </c>
     </row>
-    <row r="124" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A124" s="62" t="s">
         <v>271</v>
       </c>
@@ -15225,7 +15224,7 @@
         <v>74.74167845995774</v>
       </c>
     </row>
-    <row r="125" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A125" s="62" t="s">
         <v>272</v>
       </c>
@@ -15318,7 +15317,7 @@
         <v>14.010914448558633</v>
       </c>
     </row>
-    <row r="126" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A126" s="62" t="s">
         <v>273</v>
       </c>
@@ -15437,7 +15436,7 @@
         <v>23.87</v>
       </c>
     </row>
-    <row r="127" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A127" s="62" t="s">
         <v>274</v>
       </c>
@@ -15554,7 +15553,7 @@
         <v>1162</v>
       </c>
     </row>
-    <row r="128" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A128" s="62" t="s">
         <v>276</v>
       </c>
@@ -15673,7 +15672,7 @@
         <v>386.34994787044178</v>
       </c>
     </row>
-    <row r="129" spans="1:151" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:151" ht="18" x14ac:dyDescent="0.35">
       <c r="A129" s="62" t="s">
         <v>278</v>
       </c>
@@ -15792,7 +15791,7 @@
         <v>0.99</v>
       </c>
     </row>
-    <row r="130" spans="1:151" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:151" ht="18" x14ac:dyDescent="0.35">
       <c r="A130" s="62" t="s">
         <v>280</v>
       </c>
@@ -15911,7 +15910,7 @@
         <v>0.75934579439252337</v>
       </c>
     </row>
-    <row r="131" spans="1:151" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:151" ht="18" x14ac:dyDescent="0.35">
       <c r="A131" s="62" t="s">
         <v>282</v>
       </c>
@@ -16030,7 +16029,7 @@
         <v>4.731308411214953</v>
       </c>
     </row>
-    <row r="132" spans="1:151" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:151" ht="18" x14ac:dyDescent="0.35">
       <c r="A132" s="62" t="s">
         <v>284</v>
       </c>
@@ -16363,7 +16362,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="1:151" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:151" ht="18" x14ac:dyDescent="0.35">
       <c r="A133" s="62" t="s">
         <v>482</v>
       </c>
@@ -16752,7 +16751,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="134" spans="1:151" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:151" ht="18" x14ac:dyDescent="0.35">
       <c r="A134" s="62" t="s">
         <v>483</v>
       </c>
@@ -16799,7 +16798,7 @@
       <c r="AL134" s="15"/>
       <c r="AM134" s="15"/>
     </row>
-    <row r="135" spans="1:151" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:151" ht="18" x14ac:dyDescent="0.35">
       <c r="A135" s="62" t="s">
         <v>484</v>
       </c>
@@ -17188,7 +17187,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="136" spans="1:151" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:151" ht="18" x14ac:dyDescent="0.35">
       <c r="A136" s="62" t="s">
         <v>485</v>
       </c>
@@ -17577,7 +17576,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:151" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:151" ht="18" x14ac:dyDescent="0.35">
       <c r="A137" s="62" t="s">
         <v>285</v>
       </c>
@@ -17890,7 +17889,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="138" spans="1:151" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:151" ht="18" x14ac:dyDescent="0.35">
       <c r="A138" s="62" t="s">
         <v>482</v>
       </c>
@@ -18279,7 +18278,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="139" spans="1:151" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:151" ht="18" x14ac:dyDescent="0.35">
       <c r="A139" s="62" t="s">
         <v>483</v>
       </c>
@@ -18324,7 +18323,7 @@
       <c r="AL139" s="7"/>
       <c r="AM139" s="7"/>
     </row>
-    <row r="140" spans="1:151" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:151" ht="18" x14ac:dyDescent="0.35">
       <c r="A140" s="62" t="s">
         <v>484</v>
       </c>
@@ -18713,7 +18712,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="141" spans="1:151" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:151" ht="18" x14ac:dyDescent="0.35">
       <c r="A141" s="62" t="s">
         <v>485</v>
       </c>
@@ -19102,7 +19101,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:151" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:151" ht="18" x14ac:dyDescent="0.35">
       <c r="A142" s="62" t="s">
         <v>286</v>
       </c>
@@ -19415,7 +19414,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:151" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:151" ht="18" x14ac:dyDescent="0.35">
       <c r="A143" s="62" t="s">
         <v>482</v>
       </c>
@@ -19802,7 +19801,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="144" spans="1:151" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:151" ht="18" x14ac:dyDescent="0.35">
       <c r="A144" s="62" t="s">
         <v>483</v>
       </c>
@@ -19845,7 +19844,7 @@
       <c r="AL144" s="15"/>
       <c r="AM144" s="15"/>
     </row>
-    <row r="145" spans="1:151" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:151" ht="18" x14ac:dyDescent="0.35">
       <c r="A145" s="62" t="s">
         <v>484</v>
       </c>
@@ -20232,7 +20231,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="146" spans="1:151" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:151" ht="18" x14ac:dyDescent="0.35">
       <c r="A146" s="62" t="s">
         <v>485</v>
       </c>
@@ -20619,7 +20618,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="147" spans="1:151" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:151" ht="18" x14ac:dyDescent="0.35">
       <c r="A147" s="62" t="s">
         <v>287</v>
       </c>
@@ -21004,7 +21003,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="148" spans="1:151" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:151" ht="18" x14ac:dyDescent="0.35">
       <c r="A148" s="62" t="s">
         <v>289</v>
       </c>
@@ -21121,7 +21120,7 @@
         <v>4206.9491279299627</v>
       </c>
     </row>
-    <row r="149" spans="1:151" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:151" ht="18" x14ac:dyDescent="0.35">
       <c r="A149" s="62" t="s">
         <v>291</v>
       </c>
@@ -21238,7 +21237,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="150" spans="1:151" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:151" ht="18" x14ac:dyDescent="0.35">
       <c r="A150" s="62" t="s">
         <v>293</v>
       </c>
@@ -21355,7 +21354,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="151" spans="1:151" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:151" ht="18" x14ac:dyDescent="0.35">
       <c r="A151" s="62" t="s">
         <v>294</v>
       </c>
@@ -21454,7 +21453,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="152" spans="1:151" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:151" ht="18" x14ac:dyDescent="0.35">
       <c r="A152" s="62" t="s">
         <v>295</v>
       </c>
@@ -21497,7 +21496,7 @@
       <c r="AL152" s="15"/>
       <c r="AM152" s="15"/>
     </row>
-    <row r="153" spans="1:151" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:151" ht="18" x14ac:dyDescent="0.35">
       <c r="A153" s="62" t="s">
         <v>296</v>
       </c>
@@ -21590,7 +21589,7 @@
         <v>561.16196339803616</v>
       </c>
     </row>
-    <row r="154" spans="1:151" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:151" ht="18" x14ac:dyDescent="0.35">
       <c r="A154" s="62"/>
       <c r="B154" s="65"/>
       <c r="C154" s="5"/>
@@ -21631,7 +21630,7 @@
       <c r="AL154" s="7"/>
       <c r="AM154" s="7"/>
     </row>
-    <row r="155" spans="1:151" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:151" ht="18" x14ac:dyDescent="0.35">
       <c r="A155" s="62" t="s">
         <v>297</v>
       </c>
@@ -21688,7 +21687,7 @@
       <c r="AL155" s="7"/>
       <c r="AM155" s="7"/>
     </row>
-    <row r="156" spans="1:151" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:151" ht="18" x14ac:dyDescent="0.35">
       <c r="A156" s="62" t="s">
         <v>298</v>
       </c>
@@ -21781,7 +21780,7 @@
         <v>554.51269041060084</v>
       </c>
     </row>
-    <row r="157" spans="1:151" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:151" ht="18" x14ac:dyDescent="0.35">
       <c r="A157" s="62" t="s">
         <v>299</v>
       </c>
@@ -21874,7 +21873,7 @@
         <v>556.08738935449344</v>
       </c>
     </row>
-    <row r="158" spans="1:151" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:151" ht="18" x14ac:dyDescent="0.35">
       <c r="A158" s="62" t="s">
         <v>138</v>
       </c>
@@ -21921,7 +21920,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="159" spans="1:151" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:151" ht="18" x14ac:dyDescent="0.35">
       <c r="A159" s="62"/>
       <c r="B159" s="5" t="s">
         <v>143</v>
@@ -22038,7 +22037,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="160" spans="1:151" s="68" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:151" s="68" customFormat="1" ht="18" x14ac:dyDescent="0.35">
       <c r="A160" s="71" t="s">
         <v>301</v>
       </c>
@@ -22090,7 +22089,7 @@
       <c r="BH160" s="60"/>
       <c r="BI160" s="60"/>
     </row>
-    <row r="161" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A161" s="62" t="s">
         <v>302</v>
       </c>
@@ -22209,7 +22208,7 @@
         <v>79.603825136612031</v>
       </c>
     </row>
-    <row r="162" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A162" s="62" t="s">
         <v>304</v>
       </c>
@@ -22328,7 +22327,7 @@
         <v>90.303758366226191</v>
       </c>
     </row>
-    <row r="163" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A163" s="62" t="s">
         <v>306</v>
       </c>
@@ -22447,7 +22446,7 @@
         <v>1102.5432283695334</v>
       </c>
     </row>
-    <row r="164" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A164" s="62" t="s">
         <v>308</v>
       </c>
@@ -22566,7 +22565,7 @@
         <v>1033.3127096290989</v>
       </c>
     </row>
-    <row r="165" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A165" s="62" t="s">
         <v>309</v>
       </c>
@@ -22685,7 +22684,7 @@
         <v>69.230518740434405</v>
       </c>
     </row>
-    <row r="166" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A166" s="62" t="s">
         <v>310</v>
       </c>
@@ -22804,7 +22803,7 @@
         <v>64.443648441824877</v>
       </c>
     </row>
-    <row r="167" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A167" s="62" t="s">
         <v>311</v>
       </c>
@@ -22915,7 +22914,7 @@
         <v>24.129733954215375</v>
       </c>
     </row>
-    <row r="168" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A168" s="62" t="s">
         <v>312</v>
       </c>
@@ -23034,7 +23033,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="169" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A169" s="62" t="s">
         <v>313</v>
       </c>
@@ -23153,7 +23152,7 @@
         <v>0.85556351558175125</v>
       </c>
     </row>
-    <row r="170" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A170" s="62" t="s">
         <v>315</v>
       </c>
@@ -23272,7 +23271,7 @@
         <v>7.6036341137777201</v>
       </c>
     </row>
-    <row r="171" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A171" s="62" t="s">
         <v>316</v>
       </c>
@@ -23391,7 +23390,7 @@
         <v>12.61845061708294</v>
       </c>
     </row>
-    <row r="172" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A172" s="62" t="s">
         <v>317</v>
       </c>
@@ -23510,7 +23509,7 @@
         <v>6.6427594516265591</v>
       </c>
     </row>
-    <row r="173" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A173" s="62" t="s">
         <v>318</v>
       </c>
@@ -23629,7 +23628,7 @@
         <v>13.57199843694031</v>
       </c>
     </row>
-    <row r="174" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A174" s="62" t="s">
         <v>319</v>
       </c>
@@ -23748,7 +23747,7 @@
         <v>90.69939157658456</v>
       </c>
     </row>
-    <row r="175" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A175" s="62" t="s">
         <v>320</v>
       </c>
@@ -23867,7 +23866,7 @@
         <v>68.470457079152737</v>
       </c>
     </row>
-    <row r="176" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A176" s="62" t="s">
         <v>322</v>
       </c>
@@ -23984,7 +23983,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="177" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A177" s="62" t="s">
         <v>328</v>
       </c>
@@ -24103,7 +24102,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="178" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A178" s="62" t="s">
         <v>330</v>
       </c>
@@ -24222,7 +24221,7 @@
         <v>59.359796802240389</v>
       </c>
     </row>
-    <row r="179" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A179" s="62" t="s">
         <v>332</v>
       </c>
@@ -24341,7 +24340,7 @@
         <v>3.9860961519631841</v>
       </c>
     </row>
-    <row r="180" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A180" s="62" t="s">
         <v>333</v>
       </c>
@@ -24460,7 +24459,7 @@
         <v>3699.6544035674469</v>
       </c>
     </row>
-    <row r="181" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A181" s="62" t="s">
         <v>335</v>
       </c>
@@ -24579,7 +24578,7 @@
         <v>92.309055466950213</v>
       </c>
     </row>
-    <row r="182" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A182" s="62" t="s">
         <v>336</v>
       </c>
@@ -24698,7 +24697,7 @@
         <v>98.552542699990354</v>
       </c>
     </row>
-    <row r="183" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A183" s="62" t="s">
         <v>337</v>
       </c>
@@ -24815,7 +24814,7 @@
         <v>1.033312709629099</v>
       </c>
     </row>
-    <row r="184" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A184" s="62" t="s">
         <v>338</v>
       </c>
@@ -24908,7 +24907,7 @@
         <v>897</v>
       </c>
     </row>
-    <row r="185" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A185" s="62"/>
       <c r="B185" s="5"/>
       <c r="C185" s="72"/>
@@ -24953,7 +24952,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="186" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A186" s="62"/>
       <c r="B186" s="5" t="s">
         <v>143</v>
@@ -25070,7 +25069,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="187" spans="1:61" s="68" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:61" s="68" customFormat="1" ht="18" x14ac:dyDescent="0.35">
       <c r="A187" s="71" t="s">
         <v>340</v>
       </c>
@@ -25122,7 +25121,7 @@
       <c r="BH187" s="60"/>
       <c r="BI187" s="60"/>
     </row>
-    <row r="188" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A188" s="71" t="s">
         <v>302</v>
       </c>
@@ -25207,7 +25206,7 @@
         <v>83.564435336976331</v>
       </c>
     </row>
-    <row r="189" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A189" s="71" t="s">
         <v>304</v>
       </c>
@@ -25292,7 +25291,7 @@
         <v>96.783510210754315</v>
       </c>
     </row>
-    <row r="190" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A190" s="62" t="s">
         <v>341</v>
       </c>
@@ -25411,7 +25410,7 @@
         <v>1098.195200893774</v>
       </c>
     </row>
-    <row r="191" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A191" s="62" t="s">
         <v>308</v>
       </c>
@@ -25530,7 +25529,7 @@
         <v>1039.2422636797528</v>
       </c>
     </row>
-    <row r="192" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A192" s="62" t="s">
         <v>309</v>
       </c>
@@ -25649,7 +25648,7 @@
         <v>58.952937214021077</v>
       </c>
     </row>
-    <row r="193" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A193" s="62" t="s">
         <v>342</v>
       </c>
@@ -25768,7 +25767,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="194" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A194" s="62" t="s">
         <v>311</v>
       </c>
@@ -25887,7 +25886,7 @@
         <v>27.555840336479616</v>
       </c>
     </row>
-    <row r="195" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A195" s="62" t="s">
         <v>310</v>
       </c>
@@ -26006,7 +26005,7 @@
         <v>64.933336619267067</v>
       </c>
     </row>
-    <row r="196" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A196" s="62" t="s">
         <v>343</v>
       </c>
@@ -26101,7 +26100,7 @@
         <v>2.6474932432987486</v>
       </c>
     </row>
-    <row r="197" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A197" s="62" t="s">
         <v>344</v>
       </c>
@@ -26220,7 +26219,7 @@
         <v>0.46824555782832639</v>
       </c>
     </row>
-    <row r="198" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A198" s="62" t="s">
         <v>315</v>
       </c>
@@ -26339,7 +26338,7 @@
         <v>0.15936778634858828</v>
       </c>
     </row>
-    <row r="199" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A199" s="62" t="s">
         <v>345</v>
       </c>
@@ -26458,7 +26457,7 @@
         <v>13.481348218613171</v>
       </c>
     </row>
-    <row r="200" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A200" s="62" t="s">
         <v>317</v>
       </c>
@@ -26577,7 +26576,7 @@
         <v>3.2364771504382617</v>
       </c>
     </row>
-    <row r="201" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A201" s="62" t="s">
         <v>346</v>
       </c>
@@ -26664,7 +26663,7 @@
         <v>3.660530185408811</v>
       </c>
     </row>
-    <row r="202" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A202" s="62" t="s">
         <v>347</v>
       </c>
@@ -26781,7 +26780,7 @@
         <v>9.7981188029343382</v>
       </c>
     </row>
-    <row r="203" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A203" s="62" t="s">
         <v>348</v>
       </c>
@@ -26900,7 +26899,7 @@
         <v>91.058492987962694</v>
       </c>
     </row>
-    <row r="204" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A204" s="62" t="s">
         <v>349</v>
       </c>
@@ -27019,7 +27018,7 @@
         <v>158.0922077922078</v>
       </c>
     </row>
-    <row r="205" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A205" s="62" t="s">
         <v>322</v>
       </c>
@@ -27130,7 +27129,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="206" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A206" s="62" t="s">
         <v>328</v>
       </c>
@@ -27247,7 +27246,7 @@
         <v>7890</v>
       </c>
     </row>
-    <row r="207" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A207" s="62" t="s">
         <v>357</v>
       </c>
@@ -27366,7 +27365,7 @@
         <v>56.076693693471668</v>
       </c>
     </row>
-    <row r="208" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A208" s="62" t="s">
         <v>358</v>
       </c>
@@ -27485,7 +27484,7 @@
         <v>3.9525018278006425</v>
       </c>
     </row>
-    <row r="209" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A209" s="62" t="s">
         <v>333</v>
       </c>
@@ -27602,7 +27601,7 @@
         <v>7290.6037833635655</v>
       </c>
     </row>
-    <row r="210" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A210" s="62" t="s">
         <v>335</v>
       </c>
@@ -27719,7 +27718,7 @@
         <v>92.419383254650072</v>
       </c>
     </row>
-    <row r="211" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A211" s="62" t="s">
         <v>336</v>
       </c>
@@ -27838,7 +27837,7 @@
         <v>98.543833147952967</v>
       </c>
     </row>
-    <row r="212" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A212" s="62" t="s">
         <v>337</v>
       </c>
@@ -27955,7 +27954,7 @@
         <v>1.0392422636797529</v>
       </c>
     </row>
-    <row r="213" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A213" s="62" t="s">
         <v>359</v>
       </c>
@@ -28070,7 +28069,7 @@
         <v>949</v>
       </c>
     </row>
-    <row r="214" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A214" s="62" t="s">
         <v>361</v>
       </c>
@@ -28187,7 +28186,7 @@
         <v>3859</v>
       </c>
     </row>
-    <row r="215" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A215" s="75" t="s">
         <v>362</v>
       </c>
@@ -28280,7 +28279,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="216" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A216" s="71" t="s">
         <v>363</v>
       </c>
@@ -28323,7 +28322,7 @@
       <c r="AL216" s="5"/>
       <c r="AM216" s="5"/>
     </row>
-    <row r="217" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A217" s="62" t="s">
         <v>364</v>
       </c>
@@ -28442,7 +28441,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="218" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A218" s="62" t="s">
         <v>366</v>
       </c>
@@ -28561,7 +28560,7 @@
         <v>48886</v>
       </c>
     </row>
-    <row r="219" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A219" s="62" t="s">
         <v>367</v>
       </c>
@@ -28680,7 +28679,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="220" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A220" s="62" t="s">
         <v>368</v>
       </c>
@@ -28789,7 +28788,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="221" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A221" s="62" t="s">
         <v>369</v>
       </c>
@@ -28908,7 +28907,7 @@
         <v>91.438765808225895</v>
       </c>
     </row>
-    <row r="222" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A222" s="62" t="s">
         <v>370</v>
       </c>
@@ -29027,7 +29026,7 @@
         <v>94.005290043814483</v>
       </c>
     </row>
-    <row r="223" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A223" s="62" t="s">
         <v>371</v>
       </c>
@@ -29144,7 +29143,7 @@
         <v>5.3950980392156866</v>
       </c>
     </row>
-    <row r="224" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A224" s="62" t="s">
         <v>372</v>
       </c>
@@ -29263,7 +29262,7 @@
         <v>92.554644808743163</v>
       </c>
     </row>
-    <row r="225" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A225" s="62" t="s">
         <v>373</v>
       </c>
@@ -29382,7 +29381,7 @@
         <v>90.707011070110696</v>
       </c>
     </row>
-    <row r="226" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A226" s="62" t="s">
         <v>374</v>
       </c>
@@ -29501,7 +29500,7 @@
         <v>75.760731604126661</v>
       </c>
     </row>
-    <row r="227" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A227" s="62"/>
       <c r="B227" s="5"/>
       <c r="C227" s="72"/>
@@ -29546,7 +29545,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="228" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A228" s="62"/>
       <c r="B228" s="5" t="s">
         <v>143</v>
@@ -29663,7 +29662,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="229" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A229" s="71" t="s">
         <v>377</v>
       </c>
@@ -29706,7 +29705,7 @@
       <c r="AL229" s="5"/>
       <c r="AM229" s="5"/>
     </row>
-    <row r="230" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A230" s="62" t="s">
         <v>364</v>
       </c>
@@ -29807,7 +29806,7 @@
         <v>1302</v>
       </c>
     </row>
-    <row r="231" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A231" s="62" t="s">
         <v>378</v>
       </c>
@@ -29908,7 +29907,7 @@
         <v>111699</v>
       </c>
     </row>
-    <row r="232" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A232" s="62" t="s">
         <v>379</v>
       </c>
@@ -30009,7 +30008,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="233" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A233" s="62" t="s">
         <v>368</v>
       </c>
@@ -30110,7 +30109,7 @@
         <v>18433</v>
       </c>
     </row>
-    <row r="234" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A234" s="62" t="s">
         <v>369</v>
       </c>
@@ -30211,7 +30210,7 @@
         <v>89.207892682234373</v>
       </c>
     </row>
-    <row r="235" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A235" s="62" t="s">
         <v>370</v>
       </c>
@@ -30312,7 +30311,7 @@
         <v>89.753404378289034</v>
       </c>
     </row>
-    <row r="236" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A236" s="62" t="s">
         <v>371</v>
       </c>
@@ -30411,7 +30410,7 @@
         <v>12.19902282144845</v>
       </c>
     </row>
-    <row r="237" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A237" s="62" t="s">
         <v>372</v>
       </c>
@@ -30512,7 +30511,7 @@
         <v>92.515027322404379</v>
       </c>
     </row>
-    <row r="238" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A238" s="62" t="s">
         <v>373</v>
       </c>
@@ -30613,7 +30612,7 @@
         <v>92.832356285347245</v>
       </c>
     </row>
-    <row r="239" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A239" s="62" t="s">
         <v>374</v>
       </c>
@@ -30714,7 +30713,7 @@
         <v>140.80121526396997</v>
       </c>
     </row>
-    <row r="240" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A240" s="62"/>
       <c r="B240" s="5"/>
       <c r="C240" s="7"/>
@@ -30755,7 +30754,7 @@
       <c r="AL240" s="7"/>
       <c r="AM240" s="7"/>
     </row>
-    <row r="241" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A241" s="62"/>
       <c r="B241" s="5" t="s">
         <v>143</v>
@@ -30872,7 +30871,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="242" spans="1:61" s="68" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:61" s="68" customFormat="1" ht="18" x14ac:dyDescent="0.35">
       <c r="A242" s="69" t="s">
         <v>380</v>
       </c>
@@ -30924,7 +30923,7 @@
       <c r="BH242" s="60"/>
       <c r="BI242" s="60"/>
     </row>
-    <row r="243" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A243" s="62" t="s">
         <v>381</v>
       </c>
@@ -31005,7 +31004,7 @@
       <c r="AL243" s="15"/>
       <c r="AM243" s="15"/>
     </row>
-    <row r="244" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A244" s="62" t="s">
         <v>382</v>
       </c>
@@ -31086,7 +31085,7 @@
       <c r="AL244" s="15"/>
       <c r="AM244" s="15"/>
     </row>
-    <row r="245" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A245" s="62" t="s">
         <v>371</v>
       </c>
@@ -31167,7 +31166,7 @@
       <c r="AL245" s="15"/>
       <c r="AM245" s="15"/>
     </row>
-    <row r="246" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A246" s="62" t="s">
         <v>372</v>
       </c>
@@ -31248,7 +31247,7 @@
       <c r="AL246" s="15"/>
       <c r="AM246" s="15"/>
     </row>
-    <row r="247" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A247" s="62" t="s">
         <v>383</v>
       </c>
@@ -31329,7 +31328,7 @@
       <c r="AL247" s="15"/>
       <c r="AM247" s="15"/>
     </row>
-    <row r="248" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A248" s="62" t="s">
         <v>384</v>
       </c>
@@ -31410,7 +31409,7 @@
       <c r="AL248" s="7"/>
       <c r="AM248" s="7"/>
     </row>
-    <row r="249" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A249" s="62" t="s">
         <v>385</v>
       </c>
@@ -31491,7 +31490,7 @@
       <c r="AL249" s="15"/>
       <c r="AM249" s="15"/>
     </row>
-    <row r="250" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A250" s="62"/>
       <c r="B250" s="5" t="s">
         <v>143</v>
@@ -31608,7 +31607,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="251" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A251" s="87" t="s">
         <v>387</v>
       </c>
@@ -31651,7 +31650,7 @@
       <c r="AL251" s="5"/>
       <c r="AM251" s="5"/>
     </row>
-    <row r="252" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A252" s="62" t="s">
         <v>381</v>
       </c>
@@ -31770,7 +31769,7 @@
         <v>6.9276065119501212E-2</v>
       </c>
     </row>
-    <row r="253" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A253" s="62" t="s">
         <v>382</v>
       </c>
@@ -31889,7 +31888,7 @@
         <v>97.799799742251992</v>
       </c>
     </row>
-    <row r="254" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A254" s="62" t="s">
         <v>371</v>
       </c>
@@ -32006,7 +32005,7 @@
         <v>24.10010391409768</v>
       </c>
     </row>
-    <row r="255" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A255" s="62" t="s">
         <v>388</v>
       </c>
@@ -32125,7 +32124,7 @@
         <v>94.916666666666657</v>
       </c>
     </row>
-    <row r="256" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A256" s="62" t="s">
         <v>389</v>
       </c>
@@ -32244,7 +32243,7 @@
         <v>85.463233495012886</v>
       </c>
     </row>
-    <row r="257" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="257" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A257" s="62" t="s">
         <v>384</v>
       </c>
@@ -32363,7 +32362,7 @@
         <v>343.78905000084205</v>
       </c>
     </row>
-    <row r="258" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A258" s="62" t="s">
         <v>385</v>
       </c>
@@ -32472,7 +32471,7 @@
         <v>1.72</v>
       </c>
     </row>
-    <row r="259" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A259" s="71" t="s">
         <v>391</v>
       </c>
@@ -32515,7 +32514,7 @@
       <c r="AL259" s="5"/>
       <c r="AM259" s="5"/>
     </row>
-    <row r="260" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A260" s="62" t="s">
         <v>392</v>
       </c>
@@ -32632,7 +32631,7 @@
         <v>1.9169329073482428</v>
       </c>
     </row>
-    <row r="261" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A261" s="62" t="s">
         <v>393</v>
       </c>
@@ -32751,7 +32750,7 @@
         <v>91.938149197355997</v>
       </c>
     </row>
-    <row r="262" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A262" s="62" t="s">
         <v>394</v>
       </c>
@@ -32868,7 +32867,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="263" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A263" s="62" t="s">
         <v>372</v>
       </c>
@@ -32985,7 +32984,7 @@
         <v>39.480874316939889</v>
       </c>
     </row>
-    <row r="264" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A264" s="62" t="s">
         <v>395</v>
       </c>
@@ -33102,7 +33101,7 @@
         <v>87.370242214532865</v>
       </c>
     </row>
-    <row r="265" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A265" s="62" t="s">
         <v>396</v>
       </c>
@@ -33219,7 +33218,7 @@
         <v>15.423762376237624</v>
       </c>
     </row>
-    <row r="266" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A266" s="71" t="s">
         <v>397</v>
       </c>
@@ -33262,7 +33261,7 @@
       <c r="AL266" s="5"/>
       <c r="AM266" s="5"/>
     </row>
-    <row r="267" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A267" s="62" t="s">
         <v>392</v>
       </c>
@@ -33379,7 +33378,7 @@
         <v>0.22984731571170577</v>
       </c>
     </row>
-    <row r="268" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A268" s="62" t="s">
         <v>393</v>
       </c>
@@ -33498,7 +33497,7 @@
         <v>92.732919254658384</v>
       </c>
     </row>
-    <row r="269" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="269" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A269" s="62" t="s">
         <v>394</v>
       </c>
@@ -33617,7 +33616,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="270" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="270" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A270" s="62" t="s">
         <v>372</v>
       </c>
@@ -33734,7 +33733,7 @@
         <v>86.885245901639337</v>
       </c>
     </row>
-    <row r="271" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A271" s="62" t="s">
         <v>399</v>
       </c>
@@ -33851,7 +33850,7 @@
         <v>66.981132075471692</v>
       </c>
     </row>
-    <row r="272" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A272" s="62" t="s">
         <v>396</v>
       </c>
@@ -33968,7 +33967,7 @@
         <v>3.504694835680751</v>
       </c>
     </row>
-    <row r="273" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A273" s="62"/>
       <c r="B273" s="5"/>
       <c r="C273" s="6"/>
@@ -34009,7 +34008,7 @@
       <c r="AL273" s="15"/>
       <c r="AM273" s="94"/>
     </row>
-    <row r="274" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A274" s="95"/>
       <c r="B274" s="5"/>
       <c r="C274" s="6"/>
@@ -34052,7 +34051,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="275" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A275" s="62"/>
       <c r="B275" s="5" t="s">
         <v>143</v>
@@ -34169,7 +34168,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="276" spans="1:61" s="68" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:61" s="68" customFormat="1" ht="18" x14ac:dyDescent="0.35">
       <c r="A276" s="71" t="s">
         <v>401</v>
       </c>
@@ -34221,7 +34220,7 @@
       <c r="BH276" s="60"/>
       <c r="BI276" s="60"/>
     </row>
-    <row r="277" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A277" s="62" t="s">
         <v>402</v>
       </c>
@@ -34300,7 +34299,7 @@
       <c r="AL277" s="15"/>
       <c r="AM277" s="15"/>
     </row>
-    <row r="278" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A278" s="62" t="s">
         <v>404</v>
       </c>
@@ -34381,7 +34380,7 @@
       <c r="AL278" s="7"/>
       <c r="AM278" s="7"/>
     </row>
-    <row r="279" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A279" s="62" t="s">
         <v>406</v>
       </c>
@@ -34462,7 +34461,7 @@
       <c r="AL279" s="7"/>
       <c r="AM279" s="7"/>
     </row>
-    <row r="280" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A280" s="62" t="s">
         <v>404</v>
       </c>
@@ -34543,7 +34542,7 @@
       <c r="AL280" s="15"/>
       <c r="AM280" s="15"/>
     </row>
-    <row r="281" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A281" s="62" t="s">
         <v>406</v>
       </c>
@@ -34624,7 +34623,7 @@
       <c r="AL281" s="15"/>
       <c r="AM281" s="15"/>
     </row>
-    <row r="282" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A282" s="62" t="s">
         <v>407</v>
       </c>
@@ -34667,7 +34666,7 @@
       <c r="AL282" s="5"/>
       <c r="AM282" s="5"/>
     </row>
-    <row r="283" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A283" s="62" t="s">
         <v>408</v>
       </c>
@@ -34750,7 +34749,7 @@
       <c r="AL283" s="15"/>
       <c r="AM283" s="15"/>
     </row>
-    <row r="284" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="284" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A284" s="62" t="s">
         <v>409</v>
       </c>
@@ -34859,7 +34858,7 @@
       </c>
       <c r="AM284" s="15"/>
     </row>
-    <row r="285" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A285" s="71" t="s">
         <v>410</v>
       </c>
@@ -34902,7 +34901,7 @@
       <c r="AL285" s="5"/>
       <c r="AM285" s="5"/>
     </row>
-    <row r="286" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A286" s="62" t="s">
         <v>411</v>
       </c>
@@ -35021,7 +35020,7 @@
         <v>91.034999999999997</v>
       </c>
     </row>
-    <row r="287" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="287" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A287" s="62" t="s">
         <v>412</v>
       </c>
@@ -35138,7 +35137,7 @@
         <v>23.568341437061047</v>
       </c>
     </row>
-    <row r="288" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="288" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A288" s="62" t="s">
         <v>413</v>
       </c>
@@ -35255,7 +35254,7 @@
         <v>70.833333333333343</v>
       </c>
     </row>
-    <row r="289" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A289" s="62" t="s">
         <v>414</v>
       </c>
@@ -35372,7 +35371,7 @@
         <v>86.306653809064599</v>
       </c>
     </row>
-    <row r="290" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="290" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A290" s="62" t="s">
         <v>415</v>
       </c>
@@ -35489,7 +35488,7 @@
         <v>15.859217877094972</v>
       </c>
     </row>
-    <row r="291" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="291" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A291" s="71" t="s">
         <v>417</v>
       </c>
@@ -35532,7 +35531,7 @@
       <c r="AL291" s="5"/>
       <c r="AM291" s="5"/>
     </row>
-    <row r="292" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="292" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A292" s="62" t="s">
         <v>418</v>
       </c>
@@ -35649,7 +35648,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="293" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="293" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A293" s="62" t="s">
         <v>420</v>
       </c>
@@ -35762,7 +35761,7 @@
         <v>0.28697779450508093</v>
       </c>
     </row>
-    <row r="294" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="294" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A294" s="62" t="s">
         <v>421</v>
       </c>
@@ -35879,7 +35878,7 @@
         <v>4.3248484848484852</v>
       </c>
     </row>
-    <row r="295" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="295" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A295" s="62" t="s">
         <v>423</v>
       </c>
@@ -35996,7 +35995,7 @@
         <v>21.299868272487767</v>
       </c>
     </row>
-    <row r="296" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="296" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A296" s="71" t="s">
         <v>425</v>
       </c>
@@ -36039,7 +36038,7 @@
       <c r="AL296" s="5"/>
       <c r="AM296" s="5"/>
     </row>
-    <row r="297" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A297" s="62" t="s">
         <v>418</v>
       </c>
@@ -36156,7 +36155,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="298" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="298" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A298" s="62" t="s">
         <v>421</v>
       </c>
@@ -36273,7 +36272,7 @@
         <v>3.9214311557510793</v>
       </c>
     </row>
-    <row r="299" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="299" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A299" s="62" t="s">
         <v>423</v>
       </c>
@@ -36390,7 +36389,7 @@
         <v>21.728373589581931</v>
       </c>
     </row>
-    <row r="300" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="300" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A300" s="62"/>
       <c r="B300" s="5"/>
       <c r="C300" s="15"/>
@@ -36431,7 +36430,7 @@
       <c r="AL300" s="15"/>
       <c r="AM300" s="15"/>
     </row>
-    <row r="301" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="301" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A301" s="62"/>
       <c r="B301" s="5"/>
       <c r="C301" s="15"/>
@@ -36472,7 +36471,7 @@
       <c r="AL301" s="14"/>
       <c r="AM301" s="14"/>
     </row>
-    <row r="302" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="302" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A302" s="62"/>
       <c r="B302" s="5" t="s">
         <v>143</v>
@@ -36589,7 +36588,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="303" spans="1:61" s="68" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="303" spans="1:61" s="68" customFormat="1" ht="18" x14ac:dyDescent="0.35">
       <c r="A303" s="71" t="s">
         <v>426</v>
       </c>
@@ -36643,7 +36642,7 @@
       <c r="BH303" s="60"/>
       <c r="BI303" s="60"/>
     </row>
-    <row r="304" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="304" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A304" s="95" t="s">
         <v>427</v>
       </c>
@@ -36686,7 +36685,7 @@
       <c r="AL304" s="5"/>
       <c r="AM304" s="5"/>
     </row>
-    <row r="305" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="305" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A305" s="62" t="s">
         <v>428</v>
       </c>
@@ -36805,7 +36804,7 @@
         <v>708.23515641003132</v>
       </c>
     </row>
-    <row r="306" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="306" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A306" s="62" t="s">
         <v>430</v>
       </c>
@@ -36924,7 +36923,7 @@
         <v>599.96801612762533</v>
       </c>
     </row>
-    <row r="307" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A307" s="62" t="s">
         <v>431</v>
       </c>
@@ -37043,7 +37042,7 @@
         <v>28.034161247355637</v>
       </c>
     </row>
-    <row r="308" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="308" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A308" s="62" t="s">
         <v>432</v>
       </c>
@@ -37162,7 +37161,7 @@
         <v>20.230889604062714</v>
       </c>
     </row>
-    <row r="309" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="309" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A309" s="62" t="s">
         <v>433</v>
       </c>
@@ -37267,7 +37266,7 @@
         <v>19.078498507145049</v>
       </c>
     </row>
-    <row r="310" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="310" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A310" s="62" t="s">
         <v>434</v>
       </c>
@@ -37386,7 +37385,7 @@
         <v>356.49241827689946</v>
       </c>
     </row>
-    <row r="311" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="311" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A311" s="62" t="s">
         <v>435</v>
       </c>
@@ -37487,7 +37486,7 @@
         <v>306.50051205094144</v>
       </c>
     </row>
-    <row r="312" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="312" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A312" s="62" t="s">
         <v>436</v>
       </c>
@@ -37576,7 +37575,7 @@
       </c>
       <c r="AM312" s="7"/>
     </row>
-    <row r="313" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="313" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A313" s="62" t="s">
         <v>437</v>
       </c>
@@ -37663,7 +37662,7 @@
         <v>313.21653228317786</v>
       </c>
     </row>
-    <row r="314" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="314" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A314" s="62" t="s">
         <v>438</v>
       </c>
@@ -37782,7 +37781,7 @@
         <v>754.45068243355252</v>
       </c>
     </row>
-    <row r="315" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="315" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A315" s="62" t="s">
         <v>439</v>
       </c>
@@ -37899,7 +37898,7 @@
         <v>705.50957671152469</v>
       </c>
     </row>
-    <row r="316" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="316" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A316" s="62" t="s">
         <v>440</v>
       </c>
@@ -37944,7 +37943,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="317" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="317" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A317" s="62"/>
       <c r="B317" s="5" t="s">
         <v>143</v>
@@ -38061,7 +38060,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="318" spans="1:61" s="68" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="318" spans="1:61" s="68" customFormat="1" ht="18" x14ac:dyDescent="0.35">
       <c r="A318" s="95" t="s">
         <v>442</v>
       </c>
@@ -38113,7 +38112,7 @@
       <c r="BH318" s="60"/>
       <c r="BI318" s="60"/>
     </row>
-    <row r="319" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="319" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A319" s="62" t="s">
         <v>443</v>
       </c>
@@ -38230,7 +38229,7 @@
         <v>15.820928803441314</v>
       </c>
     </row>
-    <row r="320" spans="1:61" x14ac:dyDescent="0.35">
+    <row r="320" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A320" s="62" t="s">
         <v>445</v>
       </c>
@@ -38347,7 +38346,7 @@
         <v>65.345275613887793</v>
       </c>
     </row>
-    <row r="321" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="321" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A321" s="62" t="s">
         <v>446</v>
       </c>
@@ -38466,7 +38465,7 @@
         <v>40.200994823043409</v>
       </c>
     </row>
-    <row r="322" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="322" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A322" s="62" t="s">
         <v>447</v>
       </c>
@@ -38567,7 +38566,7 @@
         <v>38.339729895507837</v>
       </c>
     </row>
-    <row r="323" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="323" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A323" s="62" t="s">
         <v>448</v>
       </c>
@@ -38686,7 +38685,7 @@
         <v>31.246681814620374</v>
       </c>
     </row>
-    <row r="324" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="324" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A324" s="62" t="s">
         <v>449</v>
       </c>
@@ -38805,7 +38804,7 @@
         <v>41.783206708199216</v>
       </c>
     </row>
-    <row r="325" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="325" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A325" s="62" t="s">
         <v>450</v>
       </c>
@@ -38910,7 +38909,7 @@
         <v>32.193636118952682</v>
       </c>
     </row>
-    <row r="326" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="326" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A326" s="62" t="s">
         <v>451</v>
       </c>
@@ -39029,7 +39028,7 @@
         <v>141.20772411996484</v>
       </c>
     </row>
-    <row r="327" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="327" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A327" s="62" t="s">
         <v>452</v>
       </c>
@@ -39148,7 +39147,7 @@
         <v>64.337831776622224</v>
       </c>
     </row>
-    <row r="328" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="328" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A328" s="62" t="s">
         <v>453</v>
       </c>
@@ -39267,7 +39266,7 @@
         <v>74.072711671463423</v>
       </c>
     </row>
-    <row r="329" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="329" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A329" s="62" t="s">
         <v>454</v>
       </c>
@@ -39368,7 +39367,7 @@
         <v>113.13717626458045</v>
       </c>
     </row>
-    <row r="330" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="330" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A330" s="62" t="s">
         <v>455</v>
       </c>
@@ -39457,7 +39456,7 @@
       </c>
       <c r="AM330" s="15"/>
     </row>
-    <row r="331" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="331" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A331" s="62" t="s">
         <v>456</v>
       </c>
@@ -39544,7 +39543,7 @@
         <v>131.44213364945858</v>
       </c>
     </row>
-    <row r="332" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="332" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A332" s="62" t="s">
         <v>457</v>
       </c>
@@ -39663,7 +39662,7 @@
         <v>452.72818910833598</v>
       </c>
     </row>
-    <row r="333" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="333" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A333" s="71" t="s">
         <v>459</v>
       </c>
@@ -39706,7 +39705,7 @@
       <c r="AL333" s="7"/>
       <c r="AM333" s="7"/>
     </row>
-    <row r="334" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="334" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A334" s="62" t="s">
         <v>460</v>
       </c>
@@ -39823,7 +39822,7 @@
         <v>90.55</v>
       </c>
     </row>
-    <row r="335" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="335" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A335" s="62" t="s">
         <v>462</v>
       </c>
@@ -39940,7 +39939,7 @@
         <v>81.05</v>
       </c>
     </row>
-    <row r="336" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="336" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A336" s="62" t="s">
         <v>463</v>
       </c>
@@ -40057,7 +40056,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="337" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="337" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A337" s="62" t="s">
         <v>464</v>
       </c>
@@ -40174,7 +40173,7 @@
         <v>0.19500000000000001</v>
       </c>
     </row>
-    <row r="338" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="338" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A338" s="62" t="s">
         <v>465</v>
       </c>
@@ -40291,7 +40290,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="339" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="339" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A339" s="71" t="s">
         <v>466</v>
       </c>
@@ -40334,7 +40333,7 @@
       <c r="AL339" s="5"/>
       <c r="AM339" s="5"/>
     </row>
-    <row r="340" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="340" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A340" s="62" t="s">
         <v>467</v>
       </c>
@@ -40453,7 +40452,7 @@
         <v>6.1844999999999999</v>
       </c>
     </row>
-    <row r="341" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="341" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A341" s="62" t="s">
         <v>469</v>
       </c>
@@ -40572,7 +40571,7 @@
         <v>1.0386987686416256</v>
       </c>
     </row>
-    <row r="342" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="342" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A342" s="62" t="s">
         <v>470</v>
       </c>
@@ -40691,7 +40690,7 @@
         <v>1613</v>
       </c>
     </row>
-    <row r="343" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="343" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A343" s="62" t="s">
         <v>472</v>
       </c>
@@ -40810,7 +40809,7 @@
         <v>2.8750658510341411</v>
       </c>
     </row>
-    <row r="344" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="344" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A344" s="62" t="s">
         <v>472</v>
       </c>
@@ -40927,7 +40926,7 @@
         <v>2.8320737381384649</v>
       </c>
     </row>
-    <row r="345" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="345" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A345" s="62" t="s">
         <v>475</v>
       </c>
@@ -41046,7 +41045,7 @@
         <v>71.605425076603325</v>
       </c>
     </row>
-    <row r="346" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="346" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A346" s="62" t="s">
         <v>477</v>
       </c>
@@ -41109,7 +41108,7 @@
         <v>2.7349999999999999</v>
       </c>
     </row>
-    <row r="347" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="347" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A347" s="62" t="s">
         <v>479</v>
       </c>
@@ -41172,7 +41171,7 @@
         <v>554.86</v>
       </c>
     </row>
-    <row r="348" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="348" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A348" s="96" t="s">
         <v>481</v>
       </c>
@@ -41215,7 +41214,7 @@
       <c r="AL348" s="1"/>
       <c r="AM348" s="1"/>
     </row>
-    <row r="349" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="349" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A349" s="96"/>
       <c r="B349" s="1"/>
       <c r="C349" s="1"/>
@@ -41256,7 +41255,7 @@
       <c r="AL349" s="1"/>
       <c r="AM349" s="1"/>
     </row>
-    <row r="350" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="350" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A350" s="96"/>
       <c r="B350" s="1"/>
       <c r="C350" s="1"/>
@@ -41297,7 +41296,7 @@
       <c r="AL350" s="1"/>
       <c r="AM350" s="1"/>
     </row>
-    <row r="351" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="351" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A351" s="96"/>
       <c r="B351" s="1"/>
       <c r="C351" s="1"/>
@@ -41338,7 +41337,7 @@
       <c r="AL351" s="1"/>
       <c r="AM351" s="1"/>
     </row>
-    <row r="352" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="352" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A352" s="96"/>
       <c r="B352" s="1"/>
       <c r="C352" s="1"/>
@@ -41379,7 +41378,7 @@
       <c r="AL352" s="1"/>
       <c r="AM352" s="1"/>
     </row>
-    <row r="353" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="353" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A353" s="96"/>
       <c r="B353" s="1"/>
       <c r="C353" s="1"/>
@@ -41420,7 +41419,7 @@
       <c r="AL353" s="1"/>
       <c r="AM353" s="1"/>
     </row>
-    <row r="354" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="354" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A354" s="96"/>
       <c r="B354" s="1"/>
       <c r="C354" s="1"/>
@@ -41461,7 +41460,7 @@
       <c r="AL354" s="1"/>
       <c r="AM354" s="1"/>
     </row>
-    <row r="355" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="355" spans="1:39" ht="18" x14ac:dyDescent="0.35">
       <c r="A355" s="96"/>
       <c r="B355" s="1"/>
       <c r="C355" s="1"/>
@@ -41502,7 +41501,7 @@
       <c r="AL355" s="1"/>
       <c r="AM355" s="1"/>
     </row>
-    <row r="364" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="364" spans="1:39" x14ac:dyDescent="0.3">
       <c r="W364" s="98"/>
       <c r="X364" s="99"/>
       <c r="Y364" s="99"/>
@@ -41528,23 +41527,23 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A2:S49"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="18" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="18.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="38.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.6640625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="18.5546875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="38.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.7109375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="18.5703125" style="1" customWidth="1"/>
     <col min="4" max="16" width="0" style="1" hidden="1" customWidth="1"/>
-    <col min="17" max="17" width="4.6640625" style="1" hidden="1" customWidth="1"/>
-    <col min="18" max="18" width="19.6640625" style="1" customWidth="1"/>
-    <col min="19" max="16384" width="9.109375" style="2"/>
+    <col min="17" max="17" width="4.7109375" style="1" hidden="1" customWidth="1"/>
+    <col min="18" max="18" width="19.7109375" style="1" customWidth="1"/>
+    <col min="19" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:19" ht="18" x14ac:dyDescent="0.3">
       <c r="A2" s="101" t="s">
         <v>0</v>
       </c>
@@ -41554,7 +41553,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:19" ht="18" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
@@ -41578,7 +41577,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:19" ht="18" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>4</v>
       </c>
@@ -41634,7 +41633,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:19" ht="18" x14ac:dyDescent="0.3">
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
@@ -41654,7 +41653,7 @@
       <c r="Q5" s="5"/>
       <c r="R5" s="5"/>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:19" ht="18" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>22</v>
       </c>
@@ -41686,7 +41685,7 @@
         <v>89.1</v>
       </c>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:19" ht="18" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>23</v>
       </c>
@@ -41718,7 +41717,7 @@
         <v>358.8</v>
       </c>
     </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:19" ht="18" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>24</v>
       </c>
@@ -41774,7 +41773,7 @@
         <v>530.3175</v>
       </c>
     </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:19" ht="18" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
         <v>25</v>
       </c>
@@ -41810,7 +41809,7 @@
         <v>255260</v>
       </c>
     </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:19" ht="18" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
         <v>26</v>
       </c>
@@ -41846,7 +41845,7 @@
         <v>338690</v>
       </c>
     </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:19" ht="18" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
         <v>27</v>
       </c>
@@ -41882,7 +41881,7 @@
         <v>639044</v>
       </c>
     </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:19" ht="18" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
         <v>28</v>
       </c>
@@ -41938,7 +41937,7 @@
         <v>1232994</v>
       </c>
     </row>
-    <row r="13" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:19" s="1" customFormat="1" ht="18" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
         <v>29</v>
       </c>
@@ -41974,7 +41973,7 @@
         <v>171193</v>
       </c>
     </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:19" ht="18" x14ac:dyDescent="0.3">
       <c r="A14" s="8" t="s">
         <v>30</v>
       </c>
@@ -42010,7 +42009,7 @@
         <v>551046</v>
       </c>
     </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:19" ht="18" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
         <v>31</v>
       </c>
@@ -42066,7 +42065,7 @@
         <v>722239</v>
       </c>
     </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:19" ht="18" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
         <v>32</v>
       </c>
@@ -42103,7 +42102,7 @@
       </c>
       <c r="S16" s="9"/>
     </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:18" ht="18" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
         <v>33</v>
       </c>
@@ -42139,7 +42138,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:18" ht="18" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
         <v>34</v>
       </c>
@@ -42175,7 +42174,7 @@
         <v>61276</v>
       </c>
     </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:18" ht="18" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
         <v>35</v>
       </c>
@@ -42231,7 +42230,7 @@
         <v>61418</v>
       </c>
     </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:18" ht="18" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
         <v>36</v>
       </c>
@@ -42267,7 +42266,7 @@
         <v>183798</v>
       </c>
     </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:18" ht="18" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
         <v>37</v>
       </c>
@@ -42303,7 +42302,7 @@
         <v>269431</v>
       </c>
     </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
         <v>38</v>
       </c>
@@ -42339,7 +42338,7 @@
         <v>155426</v>
       </c>
     </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
         <v>39</v>
       </c>
@@ -42377,7 +42376,7 @@
         <v>608655</v>
       </c>
     </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
         <v>40</v>
       </c>
@@ -42433,7 +42432,7 @@
         <v>670073</v>
       </c>
     </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
         <v>41</v>
       </c>
@@ -42489,7 +42488,7 @@
         <v>669931</v>
       </c>
     </row>
-    <row r="26" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
         <v>42</v>
       </c>
@@ -42525,7 +42524,7 @@
         <v>408277</v>
       </c>
     </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
         <v>43</v>
       </c>
@@ -42561,7 +42560,7 @@
         <v>327931</v>
       </c>
     </row>
-    <row r="28" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
         <v>44</v>
       </c>
@@ -42597,7 +42596,7 @@
         <v>55018</v>
       </c>
     </row>
-    <row r="29" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
         <v>45</v>
       </c>
@@ -42633,7 +42632,7 @@
         <v>93116</v>
       </c>
     </row>
-    <row r="30" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A30" s="8" t="s">
         <v>46</v>
       </c>
@@ -42669,7 +42668,7 @@
         <v>177035</v>
       </c>
     </row>
-    <row r="31" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
         <v>47</v>
       </c>
@@ -42705,7 +42704,7 @@
         <v>13384</v>
       </c>
     </row>
-    <row r="32" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
         <v>48</v>
       </c>
@@ -42741,7 +42740,7 @@
         <v>7789</v>
       </c>
     </row>
-    <row r="33" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
         <v>49</v>
       </c>
@@ -42777,7 +42776,7 @@
         <v>5972</v>
       </c>
     </row>
-    <row r="34" spans="1:19" s="12" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:19" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="10" t="s">
         <v>50</v>
       </c>
@@ -42833,7 +42832,7 @@
         <v>680245</v>
       </c>
     </row>
-    <row r="35" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A35" s="13" t="s">
         <v>51</v>
       </c>
@@ -42870,7 +42869,7 @@
       </c>
       <c r="S35" s="9"/>
     </row>
-    <row r="36" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A36" s="13" t="s">
         <v>52</v>
       </c>
@@ -42902,7 +42901,7 @@
         <v>42.27</v>
       </c>
     </row>
-    <row r="37" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A37" s="13" t="s">
         <v>53</v>
       </c>
@@ -42934,7 +42933,7 @@
         <v>214.32</v>
       </c>
     </row>
-    <row r="38" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A38" s="13" t="s">
         <v>54</v>
       </c>
@@ -42966,7 +42965,7 @@
         <v>38.979999999999997</v>
       </c>
     </row>
-    <row r="39" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A39" s="13" t="s">
         <v>55</v>
       </c>
@@ -42998,7 +42997,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A40" s="13" t="s">
         <v>56</v>
       </c>
@@ -43030,7 +43029,7 @@
         <v>295.57</v>
       </c>
     </row>
-    <row r="41" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A41" s="13" t="s">
         <v>57</v>
       </c>
@@ -43062,7 +43061,7 @@
         <v>4.3</v>
       </c>
     </row>
-    <row r="42" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A42" s="10" t="s">
         <v>58</v>
       </c>
@@ -43084,7 +43083,7 @@
       <c r="Q42" s="7"/>
       <c r="R42" s="7"/>
     </row>
-    <row r="43" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A43" s="13" t="s">
         <v>59</v>
       </c>
@@ -43120,7 +43119,7 @@
         <v>2046329</v>
       </c>
     </row>
-    <row r="44" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A44" s="13" t="s">
         <v>60</v>
       </c>
@@ -43156,7 +43155,7 @@
         <v>2038129</v>
       </c>
     </row>
-    <row r="45" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A45" s="13" t="s">
         <v>61</v>
       </c>
@@ -43192,7 +43191,7 @@
         <v>159789</v>
       </c>
     </row>
-    <row r="49" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="49" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D49" s="1">
         <v>3.36</v>
       </c>
@@ -43207,33 +43206,33 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AS53"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="18" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="18.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="27.6640625" style="18" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.5546875" style="18" customWidth="1"/>
-    <col min="3" max="3" width="15.33203125" style="18" customWidth="1"/>
+    <col min="1" max="1" width="27.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5703125" style="18" customWidth="1"/>
+    <col min="3" max="3" width="15.28515625" style="18" customWidth="1"/>
     <col min="4" max="17" width="0" style="18" hidden="1" customWidth="1"/>
-    <col min="18" max="18" width="15.44140625" style="18" customWidth="1"/>
-    <col min="19" max="16384" width="9.109375" style="18"/>
+    <col min="18" max="18" width="15.42578125" style="18" customWidth="1"/>
+    <col min="19" max="16384" width="9.140625" style="18"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:45" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:45" ht="18" x14ac:dyDescent="0.3">
       <c r="A1" s="102" t="s">
         <v>62</v>
       </c>
       <c r="B1" s="102"/>
     </row>
-    <row r="2" spans="1:45" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:45" ht="18" x14ac:dyDescent="0.3">
       <c r="R2" s="18" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="3" spans="1:45" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:45" ht="18" x14ac:dyDescent="0.3">
       <c r="A3" s="7" t="s">
         <v>4</v>
       </c>
@@ -43289,7 +43288,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:45" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:45" ht="18" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
         <v>77</v>
       </c>
@@ -43311,7 +43310,7 @@
       <c r="Q4" s="7"/>
       <c r="R4" s="7"/>
     </row>
-    <row r="5" spans="1:45" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:45" ht="18" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
         <v>78</v>
       </c>
@@ -43333,7 +43332,7 @@
       <c r="Q5" s="7"/>
       <c r="R5" s="7"/>
     </row>
-    <row r="6" spans="1:45" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:45" ht="18" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
         <v>79</v>
       </c>
@@ -43369,7 +43368,7 @@
         <v>88434</v>
       </c>
     </row>
-    <row r="7" spans="1:45" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:45" ht="18" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
         <v>46</v>
       </c>
@@ -43405,7 +43404,7 @@
         <v>174554</v>
       </c>
     </row>
-    <row r="8" spans="1:45" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:45" ht="18" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
         <v>80</v>
       </c>
@@ -43441,7 +43440,7 @@
         <v>336395</v>
       </c>
     </row>
-    <row r="9" spans="1:45" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:45" ht="18" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="s">
         <v>81</v>
       </c>
@@ -43477,7 +43476,7 @@
         <v>52976</v>
       </c>
     </row>
-    <row r="10" spans="1:45" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:45" ht="18" x14ac:dyDescent="0.3">
       <c r="A10" s="7" t="s">
         <v>82</v>
       </c>
@@ -43513,7 +43512,7 @@
         <v>8319</v>
       </c>
     </row>
-    <row r="11" spans="1:45" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:45" ht="18" x14ac:dyDescent="0.3">
       <c r="A11" s="7" t="s">
         <v>83</v>
       </c>
@@ -43549,7 +43548,7 @@
         <v>5954</v>
       </c>
     </row>
-    <row r="12" spans="1:45" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:45" ht="18" x14ac:dyDescent="0.3">
       <c r="A12" s="7" t="s">
         <v>84</v>
       </c>
@@ -43581,7 +43580,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:45" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:45" ht="18" x14ac:dyDescent="0.3">
       <c r="A13" s="7" t="s">
         <v>47</v>
       </c>
@@ -43617,7 +43616,7 @@
         <v>11876</v>
       </c>
     </row>
-    <row r="14" spans="1:45" s="20" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:45" s="20" customFormat="1" ht="18" x14ac:dyDescent="0.3">
       <c r="A14" s="11" t="s">
         <v>85</v>
       </c>
@@ -43700,7 +43699,7 @@
       <c r="AR14" s="19"/>
       <c r="AS14" s="19"/>
     </row>
-    <row r="15" spans="1:45" s="19" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:45" s="19" customFormat="1" ht="18" x14ac:dyDescent="0.35">
       <c r="A15" s="7" t="s">
         <v>86</v>
       </c>
@@ -43737,7 +43736,7 @@
       </c>
       <c r="S15" s="18"/>
     </row>
-    <row r="16" spans="1:45" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:45" ht="18" x14ac:dyDescent="0.35">
       <c r="A16" s="7" t="s">
         <v>87</v>
       </c>
@@ -43773,7 +43772,7 @@
         <v>93390</v>
       </c>
     </row>
-    <row r="17" spans="1:45" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:45" ht="18" x14ac:dyDescent="0.3">
       <c r="A17" s="7" t="s">
         <v>88</v>
       </c>
@@ -43809,7 +43808,7 @@
         <v>585118</v>
       </c>
     </row>
-    <row r="18" spans="1:45" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:45" ht="18" x14ac:dyDescent="0.35">
       <c r="A18" s="7" t="s">
         <v>89</v>
       </c>
@@ -43845,7 +43844,7 @@
         <v>412682</v>
       </c>
     </row>
-    <row r="19" spans="1:45" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:45" ht="18" x14ac:dyDescent="0.35">
       <c r="A19" s="7" t="s">
         <v>90</v>
       </c>
@@ -43881,7 +43880,7 @@
         <v>704871.18</v>
       </c>
     </row>
-    <row r="20" spans="1:45" s="22" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:45" s="22" customFormat="1" ht="18" x14ac:dyDescent="0.3">
       <c r="A20" s="7" t="s">
         <v>91</v>
       </c>
@@ -43964,7 +43963,7 @@
       <c r="AR20" s="18"/>
       <c r="AS20" s="18"/>
     </row>
-    <row r="21" spans="1:45" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
         <v>92</v>
       </c>
@@ -43998,7 +43997,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:45" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A22" s="7" t="s">
         <v>93</v>
       </c>
@@ -44030,7 +44029,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:45" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
         <v>94</v>
       </c>
@@ -44062,7 +44061,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:45" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A24" s="7" t="s">
         <v>95</v>
       </c>
@@ -44094,7 +44093,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:45" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
         <v>96</v>
       </c>
@@ -44126,7 +44125,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:45" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A26" s="7" t="s">
         <v>97</v>
       </c>
@@ -44158,7 +44157,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:45" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
         <v>98</v>
       </c>
@@ -44192,7 +44191,7 @@
         <v>3288</v>
       </c>
     </row>
-    <row r="28" spans="1:45" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A28" s="7" t="s">
         <v>99</v>
       </c>
@@ -44224,7 +44223,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:45" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A29" s="7" t="s">
         <v>100</v>
       </c>
@@ -44260,7 +44259,7 @@
         <v>704</v>
       </c>
     </row>
-    <row r="30" spans="1:45" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A30" s="7" t="s">
         <v>101</v>
       </c>
@@ -44294,7 +44293,7 @@
         <v>12667</v>
       </c>
     </row>
-    <row r="31" spans="1:45" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A31" s="7" t="s">
         <v>102</v>
       </c>
@@ -44326,7 +44325,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:45" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A32" s="7" t="s">
         <v>100</v>
       </c>
@@ -44358,7 +44357,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A33" s="7" t="s">
         <v>103</v>
       </c>
@@ -44414,61 +44413,61 @@
         <v>16659</v>
       </c>
     </row>
-    <row r="34" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A34" s="23"/>
     </row>
-    <row r="35" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A35" s="23"/>
     </row>
-    <row r="36" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A36" s="23"/>
     </row>
-    <row r="37" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A37" s="23"/>
     </row>
-    <row r="38" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A38" s="23"/>
     </row>
-    <row r="39" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A39" s="23"/>
     </row>
-    <row r="40" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A40" s="23"/>
     </row>
-    <row r="41" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A41" s="23"/>
     </row>
-    <row r="42" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A42" s="23"/>
     </row>
-    <row r="43" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A43" s="23"/>
     </row>
-    <row r="44" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A44" s="23"/>
     </row>
-    <row r="45" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A45" s="23"/>
     </row>
-    <row r="46" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A46" s="23"/>
     </row>
-    <row r="47" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A47" s="23"/>
     </row>
-    <row r="48" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A48" s="23"/>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" s="23"/>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" s="24"/>
     </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" s="24"/>
     </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" s="24"/>
     </row>
   </sheetData>
@@ -44481,18 +44480,18 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:R31"/>
-  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="42.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.6640625" style="56" customWidth="1"/>
-    <col min="3" max="3" width="15.5546875" style="56" customWidth="1"/>
+    <col min="1" max="1" width="42.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.7109375" style="56" customWidth="1"/>
+    <col min="3" max="3" width="15.5703125" style="56" customWidth="1"/>
     <col min="4" max="17" width="0" style="56" hidden="1" customWidth="1"/>
-    <col min="18" max="18" width="19.33203125" style="56" customWidth="1"/>
+    <col min="18" max="18" width="19.28515625" style="56" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="18" x14ac:dyDescent="0.35">
@@ -44517,7 +44516,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:18" ht="17.45" x14ac:dyDescent="0.3">
       <c r="A2" s="33" t="s">
         <v>105</v>
       </c>
@@ -44677,7 +44676,7 @@
         <v>45.09</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A6" s="57" t="s">
         <v>109</v>
       </c>
@@ -44709,7 +44708,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:18" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:18" ht="17.45" x14ac:dyDescent="0.3">
       <c r="A7" s="44" t="s">
         <v>110</v>
       </c>
@@ -44893,7 +44892,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:18" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:18" ht="17.45" x14ac:dyDescent="0.3">
       <c r="A12" s="44" t="s">
         <v>115</v>
       </c>
@@ -45085,7 +45084,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:18" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:18" ht="17.45" x14ac:dyDescent="0.3">
       <c r="A17" s="44" t="s">
         <v>120</v>
       </c>
@@ -45269,7 +45268,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:18" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:18" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A22" s="44" t="s">
         <v>125</v>
       </c>
@@ -45325,7 +45324,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:18" ht="18" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:18" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A23" s="34" t="s">
         <v>126</v>
       </c>
@@ -45357,7 +45356,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:18" ht="18" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:18" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A24" s="34" t="s">
         <v>127</v>
       </c>
@@ -45389,7 +45388,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:18" ht="18" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:18" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A25" s="34" t="s">
         <v>128</v>
       </c>
@@ -45421,7 +45420,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:18" ht="18" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:18" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A26" s="34" t="s">
         <v>129</v>
       </c>
@@ -45455,7 +45454,7 @@
         <v>2286</v>
       </c>
     </row>
-    <row r="27" spans="1:18" ht="18" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:18" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A27" s="34" t="s">
         <v>130</v>
       </c>
@@ -45487,7 +45486,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:18" ht="18" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:18" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A28" s="34" t="s">
         <v>131</v>
       </c>
@@ -45523,7 +45522,7 @@
         <v>9547</v>
       </c>
     </row>
-    <row r="29" spans="1:18" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:18" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A29" s="44" t="s">
         <v>132</v>
       </c>
@@ -45579,7 +45578,7 @@
         <v>11833</v>
       </c>
     </row>
-    <row r="30" spans="1:18" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:18" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A30" s="44" t="s">
         <v>133</v>
       </c>
@@ -45611,7 +45610,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:18" ht="18" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:18" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A31" s="34" t="s">
         <v>134</v>
       </c>

</xml_diff>